<commit_message>
docs: Establish documentation baseline and revise co-insurance report specs
Introduces initial analysis, mapping, and rule definition documents to provide a clear baseline for the co-insurance monthly statement report project. Simultaneously, it updates the T-Account and Summary report specifications to v1.2, addressing critical discrepancies and ambiguities identified during the initial documentation phase. These revisions cover field validations, output cell locations, and calculation logic.
</commit_message>
<xml_diff>
--- a/docs/規格書/檔案位子範例/templet/PREMIUM_T_ACCOUNT.xlsx
+++ b/docs/規格書/檔案位子範例/templet/PREMIUM_T_ACCOUNT.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/64cd5bb3604bb353/Desktop/共保志工險/規格書/檔案位子範例/templet/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="66" documentId="11_AD4DBB64A54DDB1B405E389605D904C94E90DF19" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1F3976E4-A185-46B6-9655-16413E2C9D9B}"/>
+  <xr:revisionPtr revIDLastSave="72" documentId="11_AD4DBB64A54DDB1B405E389605D904C94E90DF19" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E765BAD6-9D1F-40F3-831D-321C50D8D529}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="577" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -789,22 +789,21 @@
       <c r="H20" s="8"/>
       <c r="P20" s="8"/>
     </row>
-    <row r="21" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:16" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A21" s="6"/>
       <c r="B21" t="s">
         <v>8</v>
       </c>
       <c r="H21" s="8"/>
+      <c r="O21" s="13"/>
       <c r="P21" s="8"/>
     </row>
-    <row r="22" spans="1:16" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:16" ht="16.5" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A22" s="6"/>
-      <c r="G22" s="13"/>
       <c r="H22" s="8"/>
-      <c r="O22" s="13"/>
       <c r="P22" s="8"/>
     </row>
-    <row r="23" spans="1:16" ht="16.5" thickTop="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A23" s="6"/>
       <c r="H23" s="8"/>
       <c r="P23" s="8"/>

</xml_diff>